<commit_message>
Add SavedModel folders with Git LFS
</commit_message>
<xml_diff>
--- a/reports/classification_report_random.xlsx
+++ b/reports/classification_report_random.xlsx
@@ -457,16 +457,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8666666666666667</v>
+        <v>0.4666666666666667</v>
       </c>
       <c r="C2" t="n">
-        <v>0.7222222222222222</v>
+        <v>0.28</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7878787878787878</v>
+        <v>0.35</v>
       </c>
       <c r="E2" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3">
@@ -476,16 +476,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9444444444444444</v>
+        <v>0.7222222222222222</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8095238095238095</v>
+        <v>0.5</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8717948717948718</v>
+        <v>0.5909090909090909</v>
       </c>
       <c r="E3" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4">
@@ -495,16 +495,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9285714285714286</v>
+        <v>0.35</v>
       </c>
       <c r="C4" t="n">
-        <v>0.65</v>
+        <v>0.28</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7647058823529411</v>
+        <v>0.3111111111111111</v>
       </c>
       <c r="E4" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
@@ -514,16 +514,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.9130434782608695</v>
+        <v>0.6538461538461539</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>0.6538461538461539</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9545454545454546</v>
+        <v>0.6538461538461539</v>
       </c>
       <c r="E5" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6">
@@ -533,16 +533,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.9444444444444444</v>
+        <v>0.6190476190476191</v>
       </c>
       <c r="C6" t="n">
-        <v>0.8095238095238095</v>
+        <v>0.5909090909090909</v>
       </c>
       <c r="D6" t="n">
-        <v>0.8717948717948718</v>
+        <v>0.6046511627906976</v>
       </c>
       <c r="E6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
@@ -552,16 +552,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.875</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="C7" t="n">
-        <v>0.7</v>
+        <v>0.4230769230769231</v>
       </c>
       <c r="D7" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.4888888888888889</v>
       </c>
       <c r="E7" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8">
@@ -571,16 +571,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.9</v>
+        <v>0.4482758620689655</v>
       </c>
       <c r="C8" t="n">
-        <v>0.9473684210526315</v>
+        <v>0.4814814814814815</v>
       </c>
       <c r="D8" t="n">
-        <v>0.9230769230769231</v>
+        <v>0.4642857142857143</v>
       </c>
       <c r="E8" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9">
@@ -590,16 +590,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.6818181818181818</v>
+        <v>0.28</v>
       </c>
       <c r="C9" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="D9" t="n">
-        <v>0.6976744186046512</v>
+        <v>0.2978723404255319</v>
       </c>
       <c r="E9" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10">
@@ -609,16 +609,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.9</v>
+        <v>0.65</v>
       </c>
       <c r="C10" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.8387096774193549</v>
       </c>
       <c r="D10" t="n">
-        <v>0.8780487804878049</v>
+        <v>0.7323943661971831</v>
       </c>
       <c r="E10" t="n">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11">
@@ -628,16 +628,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.8</v>
+        <v>0.4242424242424243</v>
       </c>
       <c r="C11" t="n">
-        <v>0.8</v>
+        <v>0.5185185185185185</v>
       </c>
       <c r="D11" t="n">
-        <v>0.8</v>
+        <v>0.4666666666666667</v>
       </c>
       <c r="E11" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12">
@@ -647,16 +647,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.6363636363636364</v>
+        <v>0.4736842105263158</v>
       </c>
       <c r="C12" t="n">
-        <v>0.3684210526315789</v>
+        <v>0.375</v>
       </c>
       <c r="D12" t="n">
-        <v>0.4666666666666667</v>
+        <v>0.4186046511627907</v>
       </c>
       <c r="E12" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13">
@@ -666,16 +666,16 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.35</v>
       </c>
       <c r="C13" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.5</v>
       </c>
       <c r="D13" t="n">
-        <v>0.8648648648648649</v>
+        <v>0.4117647058823529</v>
       </c>
       <c r="E13" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
@@ -685,16 +685,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="C14" t="n">
-        <v>0.631578947368421</v>
+        <v>0.3</v>
       </c>
       <c r="D14" t="n">
-        <v>0.6</v>
+        <v>0.2553191489361702</v>
       </c>
       <c r="E14" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15">
@@ -704,16 +704,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.6923076923076923</v>
       </c>
       <c r="C15" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="D15" t="n">
-        <v>0.8648648648648649</v>
+        <v>0.5806451612903226</v>
       </c>
       <c r="E15" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16">
@@ -723,16 +723,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.8235294117647058</v>
+        <v>0.4736842105263158</v>
       </c>
       <c r="C16" t="n">
-        <v>0.7</v>
+        <v>0.36</v>
       </c>
       <c r="D16" t="n">
-        <v>0.7567567567567568</v>
+        <v>0.4090909090909091</v>
       </c>
       <c r="E16" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17">
@@ -742,16 +742,16 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="C17" t="n">
-        <v>0.6</v>
+        <v>0.3461538461538461</v>
       </c>
       <c r="D17" t="n">
-        <v>0.75</v>
+        <v>0.3829787234042553</v>
       </c>
       <c r="E17" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.8125</v>
+        <v>0.3888888888888889</v>
       </c>
       <c r="C18" t="n">
-        <v>0.7222222222222222</v>
+        <v>0.2692307692307692</v>
       </c>
       <c r="D18" t="n">
-        <v>0.7647058823529411</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="E18" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19">
@@ -780,16 +780,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.6956521739130435</v>
+        <v>0.3888888888888889</v>
       </c>
       <c r="C19" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.2916666666666667</v>
       </c>
       <c r="D19" t="n">
-        <v>0.7619047619047619</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="E19" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20">
@@ -799,16 +799,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.7368421052631579</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="C20" t="n">
-        <v>0.7368421052631579</v>
+        <v>0.2142857142857143</v>
       </c>
       <c r="D20" t="n">
-        <v>0.7368421052631579</v>
+        <v>0.24</v>
       </c>
       <c r="E20" t="n">
-        <v>19</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21">
@@ -818,16 +818,16 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.5925925925925926</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="C21" t="n">
-        <v>0.8</v>
+        <v>0.5517241379310345</v>
       </c>
       <c r="D21" t="n">
-        <v>0.6808510638297872</v>
+        <v>0.5423728813559322</v>
       </c>
       <c r="E21" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22">
@@ -837,16 +837,16 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.5769230769230769</v>
+        <v>0.2619047619047619</v>
       </c>
       <c r="C22" t="n">
-        <v>0.75</v>
+        <v>0.4583333333333333</v>
       </c>
       <c r="D22" t="n">
-        <v>0.6521739130434783</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="E22" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23">
@@ -856,16 +856,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.75</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="C23" t="n">
-        <v>0.9</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="D23" t="n">
-        <v>0.8181818181818182</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="E23" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="24">
@@ -875,16 +875,16 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.8636363636363636</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="C24" t="n">
-        <v>0.8636363636363636</v>
+        <v>0.5384615384615384</v>
       </c>
       <c r="D24" t="n">
-        <v>0.8636363636363636</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="E24" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="25">
@@ -894,16 +894,16 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.2083333333333333</v>
       </c>
       <c r="C25" t="n">
-        <v>0.75</v>
+        <v>0.2272727272727273</v>
       </c>
       <c r="D25" t="n">
-        <v>0.6382978723404256</v>
+        <v>0.2173913043478261</v>
       </c>
       <c r="E25" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="26">
@@ -913,16 +913,16 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.4666666666666667</v>
       </c>
       <c r="C26" t="n">
-        <v>0.6111111111111112</v>
+        <v>0.4117647058823529</v>
       </c>
       <c r="D26" t="n">
-        <v>0.7333333333333333</v>
+        <v>0.4375</v>
       </c>
       <c r="E26" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="27">
@@ -932,16 +932,16 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.5</v>
       </c>
       <c r="C27" t="n">
-        <v>0.6</v>
+        <v>0.48</v>
       </c>
       <c r="D27" t="n">
-        <v>0.7058823529411765</v>
+        <v>0.4897959183673469</v>
       </c>
       <c r="E27" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28">
@@ -951,16 +951,16 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.6</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="C28" t="n">
-        <v>0.6818181818181818</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="D28" t="n">
-        <v>0.6382978723404256</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="E28" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="29">
@@ -970,16 +970,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.8181818181818182</v>
+        <v>0.4615384615384616</v>
       </c>
       <c r="C29" t="n">
-        <v>0.5294117647058824</v>
+        <v>0.3</v>
       </c>
       <c r="D29" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="E29" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30">
@@ -989,16 +989,16 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.8823529411764706</v>
+        <v>0.6</v>
       </c>
       <c r="C30" t="n">
-        <v>0.75</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="D30" t="n">
-        <v>0.8108108108108109</v>
+        <v>0.5</v>
       </c>
       <c r="E30" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
     </row>
     <row r="31">
@@ -1008,16 +1008,16 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.2368421052631579</v>
       </c>
       <c r="C31" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.3461538461538461</v>
       </c>
       <c r="D31" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.28125</v>
       </c>
       <c r="E31" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
     </row>
     <row r="32">
@@ -1027,16 +1027,16 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="C32" t="n">
-        <v>0.9230769230769231</v>
+        <v>0.5</v>
       </c>
       <c r="D32" t="n">
-        <v>0.7741935483870968</v>
+        <v>0.3478260869565217</v>
       </c>
       <c r="E32" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="33">
@@ -1046,16 +1046,16 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0.7647058823529411</v>
+        <v>0.5</v>
       </c>
       <c r="C33" t="n">
-        <v>0.65</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="D33" t="n">
-        <v>0.7027027027027027</v>
+        <v>0.4210526315789473</v>
       </c>
       <c r="E33" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="34">
@@ -1065,16 +1065,16 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.9047619047619048</v>
+        <v>0.9</v>
       </c>
       <c r="C34" t="n">
-        <v>0.95</v>
+        <v>0.72</v>
       </c>
       <c r="D34" t="n">
-        <v>0.926829268292683</v>
+        <v>0.8</v>
       </c>
       <c r="E34" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="35">
@@ -1084,16 +1084,16 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.72</v>
+        <v>0.625</v>
       </c>
       <c r="C35" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="D35" t="n">
-        <v>0.7826086956521739</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="E35" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
     </row>
     <row r="36">
@@ -1103,16 +1103,16 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.7083333333333334</v>
+        <v>0.4375</v>
       </c>
       <c r="C36" t="n">
-        <v>0.9444444444444444</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="D36" t="n">
-        <v>0.8095238095238095</v>
+        <v>0.3684210526315789</v>
       </c>
       <c r="E36" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="37">
@@ -1122,16 +1122,16 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="C37" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.4</v>
       </c>
       <c r="D37" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.3703703703703703</v>
       </c>
       <c r="E37" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="38">
@@ -1141,16 +1141,16 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.75</v>
       </c>
       <c r="C38" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.5454545454545454</v>
       </c>
       <c r="D38" t="n">
-        <v>0.8648648648648649</v>
+        <v>0.631578947368421</v>
       </c>
       <c r="E38" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="39">
@@ -1160,16 +1160,16 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.9444444444444444</v>
+        <v>0.4705882352941176</v>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="D39" t="n">
-        <v>0.9714285714285714</v>
+        <v>0.4324324324324325</v>
       </c>
       <c r="E39" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="40">
@@ -1179,16 +1179,16 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="D40" t="n">
-        <v>1</v>
+        <v>0.5142857142857142</v>
       </c>
       <c r="E40" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="41">
@@ -1198,16 +1198,16 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.5925925925925926</v>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>0.5925925925925926</v>
       </c>
       <c r="D41" t="n">
-        <v>0.9523809523809523</v>
+        <v>0.5925925925925926</v>
       </c>
       <c r="E41" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
     </row>
     <row r="42">
@@ -1217,16 +1217,16 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="C42" t="n">
-        <v>0.7058823529411765</v>
+        <v>0.16</v>
       </c>
       <c r="D42" t="n">
-        <v>0.7741935483870968</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="E42" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
     </row>
     <row r="43">
@@ -1236,16 +1236,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1</v>
+        <v>0.375</v>
       </c>
       <c r="C43" t="n">
-        <v>0.9444444444444444</v>
+        <v>0.36</v>
       </c>
       <c r="D43" t="n">
-        <v>0.9714285714285714</v>
+        <v>0.3673469387755102</v>
       </c>
       <c r="E43" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
     </row>
     <row r="44">
@@ -1255,16 +1255,16 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0.9473684210526315</v>
+        <v>0.68</v>
       </c>
       <c r="C44" t="n">
-        <v>0.9</v>
+        <v>0.68</v>
       </c>
       <c r="D44" t="n">
-        <v>0.9230769230769231</v>
+        <v>0.68</v>
       </c>
       <c r="E44" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="45">
@@ -1274,16 +1274,16 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.1904761904761905</v>
       </c>
       <c r="C45" t="n">
-        <v>0.7058823529411765</v>
+        <v>0.2</v>
       </c>
       <c r="D45" t="n">
-        <v>0.6857142857142857</v>
+        <v>0.1951219512195122</v>
       </c>
       <c r="E45" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="46">
@@ -1293,13 +1293,13 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.8235294117647058</v>
+        <v>0.4375</v>
       </c>
       <c r="C46" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.3888888888888889</v>
       </c>
       <c r="D46" t="n">
-        <v>0.8</v>
+        <v>0.4117647058823529</v>
       </c>
       <c r="E46" t="n">
         <v>18</v>
@@ -1312,16 +1312,16 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.7619047619047619</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="C47" t="n">
-        <v>0.7619047619047619</v>
+        <v>0.6</v>
       </c>
       <c r="D47" t="n">
-        <v>0.7619047619047619</v>
+        <v>0.5769230769230769</v>
       </c>
       <c r="E47" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="48">
@@ -1331,16 +1331,16 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0.9444444444444444</v>
+        <v>0.7222222222222222</v>
       </c>
       <c r="C48" t="n">
-        <v>0.85</v>
+        <v>0.5416666666666666</v>
       </c>
       <c r="D48" t="n">
-        <v>0.8947368421052632</v>
+        <v>0.6190476190476191</v>
       </c>
       <c r="E48" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="49">
@@ -1350,16 +1350,16 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1</v>
+        <v>0.4090909090909091</v>
       </c>
       <c r="C49" t="n">
-        <v>0.5263157894736842</v>
+        <v>0.45</v>
       </c>
       <c r="D49" t="n">
-        <v>0.6896551724137931</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="E49" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="50">
@@ -1369,13 +1369,13 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0.8947368421052632</v>
+        <v>0.4090909090909091</v>
       </c>
       <c r="C50" t="n">
-        <v>0.85</v>
+        <v>0.45</v>
       </c>
       <c r="D50" t="n">
-        <v>0.8717948717948718</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="E50" t="n">
         <v>20</v>
@@ -1388,16 +1388,16 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0.7692307692307693</v>
+        <v>0.4848484848484849</v>
       </c>
       <c r="C51" t="n">
-        <v>1</v>
+        <v>0.64</v>
       </c>
       <c r="D51" t="n">
-        <v>0.8695652173913043</v>
+        <v>0.5517241379310345</v>
       </c>
       <c r="E51" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="52">
@@ -1407,16 +1407,16 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="C52" t="n">
-        <v>0.75</v>
+        <v>0.2380952380952381</v>
       </c>
       <c r="D52" t="n">
-        <v>0.7894736842105263</v>
+        <v>0.2941176470588235</v>
       </c>
       <c r="E52" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="53">
@@ -1426,16 +1426,16 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.8947368421052632</v>
+        <v>0.5588235294117647</v>
       </c>
       <c r="C53" t="n">
-        <v>0.85</v>
+        <v>0.76</v>
       </c>
       <c r="D53" t="n">
-        <v>0.8717948717948718</v>
+        <v>0.6440677966101694</v>
       </c>
       <c r="E53" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="54">
@@ -1445,16 +1445,16 @@
         </is>
       </c>
       <c r="B54" t="n">
+        <v>0.7692307692307693</v>
+      </c>
+      <c r="C54" t="n">
         <v>0.8695652173913043</v>
       </c>
-      <c r="C54" t="n">
-        <v>1</v>
-      </c>
       <c r="D54" t="n">
-        <v>0.9302325581395349</v>
+        <v>0.8163265306122449</v>
       </c>
       <c r="E54" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="55">
@@ -1464,16 +1464,16 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0.8125</v>
+        <v>0.8</v>
       </c>
       <c r="C55" t="n">
-        <v>0.65</v>
+        <v>0.32</v>
       </c>
       <c r="D55" t="n">
-        <v>0.7222222222222222</v>
+        <v>0.4571428571428571</v>
       </c>
       <c r="E55" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="56">
@@ -1483,16 +1483,16 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="C56" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.2962962962962963</v>
       </c>
       <c r="D56" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.3265306122448979</v>
       </c>
       <c r="E56" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
     </row>
     <row r="57">
@@ -1502,16 +1502,16 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="C57" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="D57" t="n">
-        <v>0.8648648648648649</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="E57" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="58">
@@ -1521,16 +1521,16 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>0.7894736842105263</v>
+        <v>0.2702702702702703</v>
       </c>
       <c r="C58" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.4347826086956522</v>
       </c>
       <c r="D58" t="n">
-        <v>0.8108108108108109</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="E58" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
     </row>
     <row r="59">
@@ -1540,16 +1540,16 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>0.7647058823529411</v>
+        <v>0.4375</v>
       </c>
       <c r="C59" t="n">
-        <v>0.6842105263157895</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="D59" t="n">
-        <v>0.7222222222222222</v>
+        <v>0.3684210526315789</v>
       </c>
       <c r="E59" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="60">
@@ -1559,16 +1559,16 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="C60" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="D60" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.3076923076923077</v>
       </c>
       <c r="E60" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="61">
@@ -1578,16 +1578,16 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>0.9285714285714286</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="C61" t="n">
-        <v>0.7647058823529411</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="D61" t="n">
-        <v>0.8387096774193549</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E61" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="62">
@@ -1597,16 +1597,16 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>0.6842105263157895</v>
+        <v>0.1724137931034483</v>
       </c>
       <c r="C62" t="n">
-        <v>0.7222222222222222</v>
+        <v>0.25</v>
       </c>
       <c r="D62" t="n">
-        <v>0.7027027027027027</v>
+        <v>0.2040816326530612</v>
       </c>
       <c r="E62" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="63">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>0.7857142857142857</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="C63" t="n">
-        <v>0.6470588235294118</v>
+        <v>0.3043478260869565</v>
       </c>
       <c r="D63" t="n">
-        <v>0.7096774193548387</v>
+        <v>0.3111111111111111</v>
       </c>
       <c r="E63" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="64">
@@ -1635,16 +1635,16 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.2258064516129032</v>
       </c>
       <c r="C64" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="D64" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="E64" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="65">
@@ -1654,16 +1654,16 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.6842105263157895</v>
+        <v>0.375</v>
       </c>
       <c r="C65" t="n">
-        <v>0.8125</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="D65" t="n">
-        <v>0.7428571428571429</v>
+        <v>0.4</v>
       </c>
       <c r="E65" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="66">
@@ -1673,16 +1673,16 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.2380952380952381</v>
       </c>
       <c r="C66" t="n">
-        <v>0.6875</v>
+        <v>0.25</v>
       </c>
       <c r="D66" t="n">
-        <v>0.7857142857142857</v>
+        <v>0.2439024390243902</v>
       </c>
       <c r="E66" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="67">
@@ -1692,16 +1692,16 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>0.8823529411764706</v>
+        <v>0.44</v>
       </c>
       <c r="C67" t="n">
-        <v>0.7894736842105263</v>
+        <v>0.4583333333333333</v>
       </c>
       <c r="D67" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="E67" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="68">
@@ -1711,16 +1711,16 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>0.7857142857142857</v>
+        <v>0.3666666666666666</v>
       </c>
       <c r="C68" t="n">
-        <v>0.6470588235294118</v>
+        <v>0.5</v>
       </c>
       <c r="D68" t="n">
-        <v>0.7096774193548387</v>
+        <v>0.4230769230769231</v>
       </c>
       <c r="E68" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="69">
@@ -1730,16 +1730,16 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>0.85</v>
+        <v>0.2916666666666667</v>
       </c>
       <c r="C69" t="n">
-        <v>0.85</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="D69" t="n">
-        <v>0.85</v>
+        <v>0.3111111111111111</v>
       </c>
       <c r="E69" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="70">
@@ -1749,16 +1749,16 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>0.9375</v>
+        <v>0.75</v>
       </c>
       <c r="C70" t="n">
-        <v>0.8823529411764706</v>
+        <v>0.5</v>
       </c>
       <c r="D70" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.6</v>
       </c>
       <c r="E70" t="n">
-        <v>17</v>
+        <v>30</v>
       </c>
     </row>
     <row r="71">
@@ -1768,16 +1768,16 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>1</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="C71" t="n">
-        <v>0.6842105263157895</v>
+        <v>0.3076923076923077</v>
       </c>
       <c r="D71" t="n">
-        <v>0.8125</v>
+        <v>0.4</v>
       </c>
       <c r="E71" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
     </row>
     <row r="72">
@@ -1787,16 +1787,16 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="C72" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.6111111111111112</v>
       </c>
       <c r="D72" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.5945945945945946</v>
       </c>
       <c r="E72" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="73">
@@ -1806,16 +1806,16 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>0.875</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="C73" t="n">
-        <v>0.8235294117647058</v>
+        <v>0.5</v>
       </c>
       <c r="D73" t="n">
-        <v>0.8484848484848485</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="E73" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="74">
@@ -1825,13 +1825,13 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>0.6111111111111112</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="C74" t="n">
-        <v>0.55</v>
+        <v>0.3</v>
       </c>
       <c r="D74" t="n">
-        <v>0.5789473684210527</v>
+        <v>0.3243243243243243</v>
       </c>
       <c r="E74" t="n">
         <v>20</v>
@@ -1844,16 +1844,16 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>1</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="C75" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="D75" t="n">
-        <v>0.875</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="E75" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="76">
@@ -1863,16 +1863,16 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>0.7272727272727273</v>
+        <v>0.5238095238095238</v>
       </c>
       <c r="C76" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.44</v>
       </c>
       <c r="D76" t="n">
-        <v>0.8205128205128205</v>
+        <v>0.4782608695652174</v>
       </c>
       <c r="E76" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
     </row>
     <row r="77">
@@ -1882,16 +1882,16 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>0.8235294117647058</v>
+        <v>0.5454545454545454</v>
       </c>
       <c r="C77" t="n">
-        <v>0.7</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="D77" t="n">
-        <v>0.7567567567567568</v>
+        <v>0.4897959183673469</v>
       </c>
       <c r="E77" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
     </row>
     <row r="78">
@@ -1901,16 +1901,16 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>0.8125</v>
+        <v>0.4615384615384616</v>
       </c>
       <c r="C78" t="n">
-        <v>0.7222222222222222</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="D78" t="n">
-        <v>0.7647058823529411</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="E78" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="79">
@@ -1920,16 +1920,16 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.6470588235294118</v>
       </c>
       <c r="C79" t="n">
-        <v>0.8</v>
+        <v>0.44</v>
       </c>
       <c r="D79" t="n">
-        <v>0.8648648648648649</v>
+        <v>0.5238095238095238</v>
       </c>
       <c r="E79" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="80">
@@ -1939,16 +1939,16 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>0.7727272727272727</v>
+        <v>0.4571428571428571</v>
       </c>
       <c r="C80" t="n">
-        <v>0.8947368421052632</v>
+        <v>0.6153846153846154</v>
       </c>
       <c r="D80" t="n">
-        <v>0.8292682926829268</v>
+        <v>0.5245901639344263</v>
       </c>
       <c r="E80" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
     </row>
     <row r="81">
@@ -1958,16 +1958,16 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>0.6538461538461539</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="C81" t="n">
-        <v>0.85</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="D81" t="n">
-        <v>0.7391304347826086</v>
+        <v>0.3934426229508197</v>
       </c>
       <c r="E81" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
     </row>
     <row r="82">
@@ -1977,16 +1977,16 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>0.8181818181818182</v>
+        <v>0.5294117647058824</v>
       </c>
       <c r="C82" t="n">
-        <v>0.9473684210526315</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="D82" t="n">
-        <v>0.8780487804878049</v>
+        <v>0.4090909090909091</v>
       </c>
       <c r="E82" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
     </row>
     <row r="83">
@@ -1996,16 +1996,16 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0.85</v>
+        <v>0.68</v>
       </c>
       <c r="C83" t="n">
-        <v>0.8947368421052632</v>
+        <v>0.7391304347826086</v>
       </c>
       <c r="D83" t="n">
-        <v>0.8717948717948718</v>
+        <v>0.7083333333333334</v>
       </c>
       <c r="E83" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="84">
@@ -2015,16 +2015,16 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>0.9</v>
+        <v>0.4705882352941176</v>
       </c>
       <c r="C84" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="D84" t="n">
-        <v>0.8780487804878049</v>
+        <v>0.4102564102564102</v>
       </c>
       <c r="E84" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="85">
@@ -2034,16 +2034,16 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>0.9230769230769231</v>
+        <v>0.391304347826087</v>
       </c>
       <c r="C85" t="n">
-        <v>0.631578947368421</v>
+        <v>0.36</v>
       </c>
       <c r="D85" t="n">
-        <v>0.75</v>
+        <v>0.375</v>
       </c>
       <c r="E85" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
     <row r="86">
@@ -2053,16 +2053,16 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>0.9047619047619048</v>
+        <v>0.5769230769230769</v>
       </c>
       <c r="C86" t="n">
-        <v>0.95</v>
+        <v>0.625</v>
       </c>
       <c r="D86" t="n">
-        <v>0.926829268292683</v>
+        <v>0.6</v>
       </c>
       <c r="E86" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="87">
@@ -2072,16 +2072,16 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.2352941176470588</v>
       </c>
       <c r="C87" t="n">
-        <v>0.4210526315789473</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="D87" t="n">
-        <v>0.4848484848484849</v>
+        <v>0.2285714285714286</v>
       </c>
       <c r="E87" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="88">
@@ -2091,16 +2091,16 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>0.4545454545454545</v>
+        <v>0.1590909090909091</v>
       </c>
       <c r="C88" t="n">
-        <v>0.7894736842105263</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="D88" t="n">
-        <v>0.5769230769230769</v>
+        <v>0.2121212121212121</v>
       </c>
       <c r="E88" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="89">
@@ -2110,16 +2110,16 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>0.9473684210526315</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="C89" t="n">
-        <v>0.9473684210526315</v>
+        <v>0.48</v>
       </c>
       <c r="D89" t="n">
-        <v>0.9473684210526315</v>
+        <v>0.4528301886792453</v>
       </c>
       <c r="E89" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
     <row r="90">
@@ -2129,16 +2129,16 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>0.7692307692307693</v>
+        <v>0.5217391304347826</v>
       </c>
       <c r="C90" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="D90" t="n">
         <v>0.5</v>
       </c>
-      <c r="D90" t="n">
-        <v>0.6060606060606061</v>
-      </c>
       <c r="E90" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="91">
@@ -2148,16 +2148,16 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>0.8636363636363636</v>
+        <v>0.65625</v>
       </c>
       <c r="C91" t="n">
-        <v>0.95</v>
+        <v>0.8076923076923077</v>
       </c>
       <c r="D91" t="n">
-        <v>0.9047619047619048</v>
+        <v>0.7241379310344828</v>
       </c>
       <c r="E91" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="92">
@@ -2167,16 +2167,16 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>0.7058823529411765</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="C92" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.1923076923076923</v>
       </c>
       <c r="D92" t="n">
-        <v>0.6857142857142857</v>
+        <v>0.1785714285714286</v>
       </c>
       <c r="E92" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
     <row r="93">
@@ -2186,13 +2186,13 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>0.8095238095238095</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="C93" t="n">
-        <v>0.85</v>
+        <v>0.75</v>
       </c>
       <c r="D93" t="n">
-        <v>0.8292682926829268</v>
+        <v>0.7317073170731707</v>
       </c>
       <c r="E93" t="n">
         <v>20</v>
@@ -2205,16 +2205,16 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>0.8235294117647058</v>
+        <v>0.4</v>
       </c>
       <c r="C94" t="n">
-        <v>0.8235294117647058</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="D94" t="n">
-        <v>0.8235294117647058</v>
+        <v>0.4210526315789473</v>
       </c>
       <c r="E94" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
     </row>
     <row r="95">
@@ -2224,16 +2224,16 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>0.75</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="C95" t="n">
-        <v>0.631578947368421</v>
+        <v>0.2</v>
       </c>
       <c r="D95" t="n">
-        <v>0.6857142857142857</v>
+        <v>0.2564102564102564</v>
       </c>
       <c r="E95" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
     <row r="96">
@@ -2243,13 +2243,13 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.3125</v>
       </c>
       <c r="C96" t="n">
-        <v>0.7692307692307693</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="D96" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="E96" t="n">
         <v>13</v>
@@ -2262,16 +2262,16 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>0.9473684210526315</v>
+        <v>0.375</v>
       </c>
       <c r="C97" t="n">
-        <v>1</v>
+        <v>0.4090909090909091</v>
       </c>
       <c r="D97" t="n">
-        <v>0.972972972972973</v>
+        <v>0.391304347826087</v>
       </c>
       <c r="E97" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="98">
@@ -2281,16 +2281,16 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>0.9473684210526315</v>
+        <v>0.7619047619047619</v>
       </c>
       <c r="C98" t="n">
-        <v>1</v>
+        <v>0.6956521739130435</v>
       </c>
       <c r="D98" t="n">
-        <v>0.972972972972973</v>
+        <v>0.7272727272727273</v>
       </c>
       <c r="E98" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
     </row>
     <row r="99">
@@ -2300,16 +2300,16 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.3684210526315789</v>
       </c>
       <c r="C99" t="n">
-        <v>0.75</v>
+        <v>0.3043478260869565</v>
       </c>
       <c r="D99" t="n">
-        <v>0.7894736842105263</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="E99" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="100">
@@ -2319,16 +2319,16 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>0.7368421052631579</v>
+        <v>0.3870967741935484</v>
       </c>
       <c r="C100" t="n">
-        <v>0.8235294117647058</v>
+        <v>0.4615384615384616</v>
       </c>
       <c r="D100" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.4210526315789473</v>
       </c>
       <c r="E100" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
     </row>
     <row r="101">
@@ -2338,16 +2338,16 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="C101" t="n">
-        <v>0.8235294117647058</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="D101" t="n">
-        <v>0.8</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="E101" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="102">
@@ -2357,16 +2357,16 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>0.6551724137931034</v>
+        <v>0.44</v>
       </c>
       <c r="C102" t="n">
-        <v>1</v>
+        <v>0.55</v>
       </c>
       <c r="D102" t="n">
-        <v>0.7916666666666666</v>
+        <v>0.4888888888888889</v>
       </c>
       <c r="E102" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="103">
@@ -2376,16 +2376,16 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>0.875</v>
+        <v>0.5925925925925926</v>
       </c>
       <c r="C103" t="n">
-        <v>0.7368421052631579</v>
+        <v>0.6153846153846154</v>
       </c>
       <c r="D103" t="n">
-        <v>0.8</v>
+        <v>0.6037735849056604</v>
       </c>
       <c r="E103" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
     </row>
     <row r="104">
@@ -2395,16 +2395,16 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>0.9375</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="C104" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="D104" t="n">
-        <v>0.8823529411764706</v>
+        <v>0.2162162162162162</v>
       </c>
       <c r="E104" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
     <row r="105">
@@ -2414,16 +2414,16 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="C105" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.2083333333333333</v>
       </c>
       <c r="D105" t="n">
-        <v>0.8648648648648649</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="E105" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="106">
@@ -2433,16 +2433,16 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.2380952380952381</v>
       </c>
       <c r="C106" t="n">
-        <v>0.5263157894736842</v>
+        <v>0.25</v>
       </c>
       <c r="D106" t="n">
-        <v>0.5882352941176471</v>
+        <v>0.2439024390243902</v>
       </c>
       <c r="E106" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="107">
@@ -2452,16 +2452,16 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>0.9444444444444444</v>
+        <v>0.7222222222222222</v>
       </c>
       <c r="C107" t="n">
-        <v>0.85</v>
+        <v>0.5</v>
       </c>
       <c r="D107" t="n">
-        <v>0.8947368421052632</v>
+        <v>0.5909090909090909</v>
       </c>
       <c r="E107" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="108">
@@ -2471,16 +2471,16 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>0.46875</v>
+        <v>0.3548387096774194</v>
       </c>
       <c r="C108" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.4782608695652174</v>
       </c>
       <c r="D108" t="n">
-        <v>0.6</v>
+        <v>0.4074074074074074</v>
       </c>
       <c r="E108" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
     </row>
     <row r="109">
@@ -2490,16 +2490,16 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.6875</v>
       </c>
       <c r="C109" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.7857142857142857</v>
       </c>
       <c r="D109" t="n">
-        <v>0.8648648648648649</v>
+        <v>0.7333333333333333</v>
       </c>
       <c r="E109" t="n">
-        <v>19</v>
+        <v>28</v>
       </c>
     </row>
     <row r="110">
@@ -2509,16 +2509,16 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>0.6521739130434783</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="C110" t="n">
-        <v>0.8823529411764706</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="D110" t="n">
-        <v>0.75</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="E110" t="n">
-        <v>17</v>
+        <v>28</v>
       </c>
     </row>
     <row r="111">
@@ -2528,16 +2528,16 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>0.5652173913043478</v>
+        <v>0.4814814814814815</v>
       </c>
       <c r="C111" t="n">
-        <v>0.6190476190476191</v>
+        <v>0.5</v>
       </c>
       <c r="D111" t="n">
-        <v>0.5909090909090909</v>
+        <v>0.4905660377358491</v>
       </c>
       <c r="E111" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="112">
@@ -2547,16 +2547,16 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>0.6153846153846154</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="C112" t="n">
-        <v>0.8</v>
+        <v>0.6086956521739131</v>
       </c>
       <c r="D112" t="n">
-        <v>0.6956521739130435</v>
+        <v>0.3888888888888889</v>
       </c>
       <c r="E112" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="113">
@@ -2566,16 +2566,16 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>0.8</v>
+        <v>0.48</v>
       </c>
       <c r="C113" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.5</v>
       </c>
       <c r="D113" t="n">
-        <v>0.8205128205128205</v>
+        <v>0.4897959183673469</v>
       </c>
       <c r="E113" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="114">
@@ -2585,16 +2585,16 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="C114" t="n">
-        <v>0.6842105263157895</v>
+        <v>0.25</v>
       </c>
       <c r="D114" t="n">
-        <v>0.5777777777777777</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="E114" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="115">
@@ -2604,16 +2604,16 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>0.7647058823529411</v>
+        <v>0.2</v>
       </c>
       <c r="C115" t="n">
-        <v>0.6842105263157895</v>
+        <v>0.1153846153846154</v>
       </c>
       <c r="D115" t="n">
-        <v>0.7222222222222222</v>
+        <v>0.1463414634146341</v>
       </c>
       <c r="E115" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
     </row>
     <row r="116">
@@ -2623,16 +2623,16 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>0.625</v>
+        <v>0.16</v>
       </c>
       <c r="C116" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.2</v>
       </c>
       <c r="D116" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.1777777777777778</v>
       </c>
       <c r="E116" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="117">
@@ -2642,16 +2642,16 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.36</v>
       </c>
       <c r="C117" t="n">
-        <v>0.5789473684210527</v>
+        <v>0.45</v>
       </c>
       <c r="D117" t="n">
-        <v>0.7096774193548387</v>
+        <v>0.4</v>
       </c>
       <c r="E117" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="118">
@@ -2661,16 +2661,16 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>0.6956521739130435</v>
+        <v>0.2142857142857143</v>
       </c>
       <c r="C118" t="n">
-        <v>0.8</v>
+        <v>0.375</v>
       </c>
       <c r="D118" t="n">
-        <v>0.7441860465116279</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="E118" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
     </row>
     <row r="119">
@@ -2680,16 +2680,16 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="C119" t="n">
-        <v>0.5263157894736842</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="D119" t="n">
-        <v>0.6060606060606061</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="E119" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="120">
@@ -2699,16 +2699,16 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>0.8</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="C120" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.2142857142857143</v>
       </c>
       <c r="D120" t="n">
-        <v>0.8648648648648649</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="E120" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="121">
@@ -2718,16 +2718,16 @@
         </is>
       </c>
       <c r="B121" t="n">
-        <v>0.7647058823529411</v>
+        <v>0.2173913043478261</v>
       </c>
       <c r="C121" t="n">
-        <v>0.7222222222222222</v>
+        <v>0.2272727272727273</v>
       </c>
       <c r="D121" t="n">
-        <v>0.7428571428571429</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="E121" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="122">
@@ -2737,16 +2737,16 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>0.8095238095238095</v>
+        <v>0.6470588235294118</v>
       </c>
       <c r="C122" t="n">
-        <v>0.8095238095238095</v>
+        <v>0.4583333333333333</v>
       </c>
       <c r="D122" t="n">
-        <v>0.8095238095238095</v>
+        <v>0.5365853658536586</v>
       </c>
       <c r="E122" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="123">
@@ -2756,16 +2756,16 @@
         </is>
       </c>
       <c r="B123" t="n">
-        <v>0.9375</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="C123" t="n">
-        <v>0.8823529411764706</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="D123" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.6086956521739131</v>
       </c>
       <c r="E123" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
     </row>
     <row r="124">
@@ -2775,13 +2775,13 @@
         </is>
       </c>
       <c r="B124" t="n">
-        <v>0.8823529411764706</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="C124" t="n">
-        <v>0.6818181818181818</v>
+        <v>0.4545454545454545</v>
       </c>
       <c r="D124" t="n">
-        <v>0.7692307692307693</v>
+        <v>0.4</v>
       </c>
       <c r="E124" t="n">
         <v>22</v>
@@ -2794,16 +2794,16 @@
         </is>
       </c>
       <c r="B125" t="n">
-        <v>0.8823529411764706</v>
+        <v>0.4347826086956522</v>
       </c>
       <c r="C125" t="n">
-        <v>0.7894736842105263</v>
+        <v>0.4</v>
       </c>
       <c r="D125" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="E125" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
     <row r="126">
@@ -2813,16 +2813,16 @@
         </is>
       </c>
       <c r="B126" t="n">
-        <v>0.8636363636363636</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="C126" t="n">
-        <v>1</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="D126" t="n">
-        <v>0.926829268292683</v>
+        <v>0.5957446808510638</v>
       </c>
       <c r="E126" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
     <row r="127">
@@ -2832,16 +2832,16 @@
         </is>
       </c>
       <c r="B127" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.5862068965517241</v>
       </c>
       <c r="C127" t="n">
-        <v>0.8</v>
+        <v>0.6296296296296297</v>
       </c>
       <c r="D127" t="n">
-        <v>0.8205128205128205</v>
+        <v>0.6071428571428571</v>
       </c>
       <c r="E127" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
     </row>
     <row r="128">
@@ -2851,16 +2851,16 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="C128" t="n">
-        <v>0.8</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="D128" t="n">
-        <v>0.7272727272727273</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="E128" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="129">
@@ -2870,16 +2870,16 @@
         </is>
       </c>
       <c r="B129" t="n">
-        <v>0.4838709677419355</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="C129" t="n">
-        <v>0.8823529411764706</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="D129" t="n">
-        <v>0.625</v>
+        <v>0.16</v>
       </c>
       <c r="E129" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="130">
@@ -2889,16 +2889,16 @@
         </is>
       </c>
       <c r="B130" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.3703703703703703</v>
       </c>
       <c r="C130" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.4</v>
       </c>
       <c r="D130" t="n">
-        <v>0.6060606060606061</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="E130" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
     </row>
     <row r="131">
@@ -2908,16 +2908,16 @@
         </is>
       </c>
       <c r="B131" t="n">
-        <v>0.7333333333333333</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="C131" t="n">
-        <v>0.6111111111111112</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="D131" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.2790697674418605</v>
       </c>
       <c r="E131" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
     <row r="132">
@@ -2927,16 +2927,16 @@
         </is>
       </c>
       <c r="B132" t="n">
-        <v>0.6842105263157895</v>
+        <v>0.28</v>
       </c>
       <c r="C132" t="n">
-        <v>0.7647058823529411</v>
+        <v>0.28</v>
       </c>
       <c r="D132" t="n">
-        <v>0.7222222222222222</v>
+        <v>0.28</v>
       </c>
       <c r="E132" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
     </row>
     <row r="133">
@@ -2946,16 +2946,16 @@
         </is>
       </c>
       <c r="B133" t="n">
-        <v>0.9523809523809523</v>
+        <v>0.5757575757575758</v>
       </c>
       <c r="C133" t="n">
-        <v>0.9523809523809523</v>
+        <v>0.7916666666666666</v>
       </c>
       <c r="D133" t="n">
-        <v>0.9523809523809523</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E133" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="134">
@@ -2965,16 +2965,16 @@
         </is>
       </c>
       <c r="B134" t="n">
-        <v>0.6875</v>
+        <v>0.2142857142857143</v>
       </c>
       <c r="C134" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.1304347826086956</v>
       </c>
       <c r="D134" t="n">
-        <v>0.5945945945945946</v>
+        <v>0.1621621621621622</v>
       </c>
       <c r="E134" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="135">
@@ -2984,16 +2984,16 @@
         </is>
       </c>
       <c r="B135" t="n">
-        <v>0.85</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="C135" t="n">
-        <v>0.8947368421052632</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="D135" t="n">
-        <v>0.8717948717948718</v>
+        <v>0.3703703703703703</v>
       </c>
       <c r="E135" t="n">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="136">
@@ -3003,16 +3003,16 @@
         </is>
       </c>
       <c r="B136" t="n">
-        <v>0.68</v>
+        <v>0.4722222222222222</v>
       </c>
       <c r="C136" t="n">
-        <v>0.8947368421052632</v>
+        <v>0.5666666666666667</v>
       </c>
       <c r="D136" t="n">
-        <v>0.7727272727272727</v>
+        <v>0.5151515151515151</v>
       </c>
       <c r="E136" t="n">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="137">
@@ -3022,16 +3022,16 @@
         </is>
       </c>
       <c r="B137" t="n">
-        <v>0.786833855799373</v>
+        <v>0.4312599681020733</v>
       </c>
       <c r="C137" t="n">
-        <v>0.786833855799373</v>
+        <v>0.4312599681020733</v>
       </c>
       <c r="D137" t="n">
-        <v>0.786833855799373</v>
+        <v>0.4312599681020733</v>
       </c>
       <c r="E137" t="n">
-        <v>0.786833855799373</v>
+        <v>0.4312599681020733</v>
       </c>
     </row>
     <row r="138">
@@ -3041,16 +3041,16 @@
         </is>
       </c>
       <c r="B138" t="n">
-        <v>0.8034085294419562</v>
+        <v>0.44112218400592</v>
       </c>
       <c r="C138" t="n">
-        <v>0.7876923910601241</v>
+        <v>0.4260198196976011</v>
       </c>
       <c r="D138" t="n">
-        <v>0.7871114328825688</v>
+        <v>0.4242509066752263</v>
       </c>
       <c r="E138" t="n">
-        <v>2552</v>
+        <v>3135</v>
       </c>
     </row>
     <row r="139">
@@ -3060,16 +3060,16 @@
         </is>
       </c>
       <c r="B139" t="n">
-        <v>0.8038774251785799</v>
+        <v>0.4521323082207311</v>
       </c>
       <c r="C139" t="n">
-        <v>0.786833855799373</v>
+        <v>0.4312599681020733</v>
       </c>
       <c r="D139" t="n">
-        <v>0.7870149129488078</v>
+        <v>0.4323950325234824</v>
       </c>
       <c r="E139" t="n">
-        <v>2552</v>
+        <v>3135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>